<commit_message>
Working on getting item domain and records set in stone before moving to ordering
</commit_message>
<xml_diff>
--- a/WorkBot/main/data/orders/Webstaurant/Webstaurant_Bakery_20260524.xlsx
+++ b/WorkBot/main/data/orders/Webstaurant/Webstaurant_Bakery_20260524.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -542,6 +542,132 @@
         <v>299.52</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>433SLINERBL</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Sheet Pan Liner - Silicone Coated</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>4</v>
+      </c>
+      <c r="D9" t="n">
+        <v>84.23</v>
+      </c>
+      <c r="E9" t="n">
+        <v>336.92</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>500CTOUT160</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Java Box (160oz)</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" t="n">
+        <v>100.99</v>
+      </c>
+      <c r="E10" t="n">
+        <v>201.98</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>245CCGR1914</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Cake Board - 1/2 Sheet</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>2</v>
+      </c>
+      <c r="D11" t="n">
+        <v>39.99</v>
+      </c>
+      <c r="E11" t="n">
+        <v>79.98</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>150300865</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Bag Paper - 6x13.5 Window</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D12" t="n">
+        <v>79.98999999999999</v>
+      </c>
+      <c r="E12" t="n">
+        <v>159.98</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>433qlinerbl</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Sheet Pan Liner - White</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" t="n">
+        <v>46.99</v>
+      </c>
+      <c r="E13" t="n">
+        <v>93.98</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>5004CAFE</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Cup - Espresso (4oz)</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" t="n">
+        <v>36.49</v>
+      </c>
+      <c r="E14" t="n">
+        <v>36.49</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>